<commit_message>
metas octubre 2026: M1.1 20.000→8.000, M9 10.000→8.000 (total 61.060)
Colchones con p90 de septiembre: M1.1 669 m³/día (volteo 10.007 / madereo 9.338),
M9 370 m³/día (volteo 9.110 / madereo 8.740). Fallbacks de los 6 scripts alineados
al Excel. generar_snapshots.py no se toca (solo meses cerrados).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dashboard_CosechaForestal.xlsx
+++ b/Dashboard_CosechaForestal.xlsx
@@ -17304,7 +17304,7 @@
         </is>
       </c>
       <c r="E24" s="106" t="n">
-        <v>20000</v>
+        <v>8000</v>
       </c>
       <c r="F24" s="107">
         <f>IF(CONFIGURACIÓN!$C$10=0,0,ROUND(E24/CONFIGURACIÓN!$C$10,1))</f>
@@ -17320,13 +17320,13 @@
         </is>
       </c>
       <c r="I24" s="106" t="n">
-        <v>21608</v>
+        <v>10007</v>
       </c>
       <c r="J24" s="106" t="n">
-        <v>21072</v>
+        <v>9338</v>
       </c>
       <c r="K24" s="106" t="n">
-        <v>20000</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="25" ht="19.5" customHeight="1" s="150">
@@ -17556,7 +17556,7 @@
         </is>
       </c>
       <c r="E30" s="106" t="n">
-        <v>10000</v>
+        <v>8000</v>
       </c>
       <c r="F30" s="107">
         <f>IF(CONFIGURACIÓN!$C$10=0,0,ROUND(E30/CONFIGURACIÓN!$C$10,1))</f>
@@ -17572,13 +17572,13 @@
         </is>
       </c>
       <c r="I30" s="106" t="n">
-        <v>10939</v>
+        <v>9110</v>
       </c>
       <c r="J30" s="106" t="n">
-        <v>10626</v>
+        <v>8740</v>
       </c>
       <c r="K30" s="106" t="n">
-        <v>10000</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="31" ht="19.5" customHeight="1" s="150">

</xml_diff>